<commit_message>
docs: update Scrum evidence for HU-023 and HU-024
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Grupales/06_Product_Backlog_CitaJusta.xlsx
+++ b/Fase 2/Evidencias Grupales/06_Product_Backlog_CitaJusta.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Backlog" sheetId="1" r:id="R22981fd68d2c4db4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="Rcd99e25ae9ae403e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Backlog" sheetId="1" r:id="R92565426a82e4bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="Rc72a9f3989734803"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -693,7 +693,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -763,6 +763,72 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1063,7 +1129,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd891750588d94096"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf2214246ca274b20"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1325,7 +1391,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="10" t="str">
-        <x:v>Versión 1.5 · Actualización 20-09-2026 · Backend HU-001 a HU-020 completado · HU-021 Web Done · HU-022 cierre técnico completado y validado · PR #89 mergeado.</x:v>
+        <x:v>Versión 1.6 · Actualización 21-09-2026 · Backend HU-001 a HU-020 completado · HU-021 a HU-024 Done · Sprint 6 cerrado con expiración automática y notificaciones internas.</x:v>
       </x:c>
       <x:c r="B2" s="11"/>
       <x:c r="C2" s="11"/>
@@ -2341,53 +2407,124 @@
         <x:v>MVP</x:v>
       </x:c>
       <x:c r="K26" t="str">
-        <x:v>La Web muestra ofertas reales y su expiresAt. • Permite aceptar/rechazar mediante endpoints existentes. • No calcula ranking ni elegibilidad. • Maneja expiración, conflictos y doble submit.</x:v>
+        <x:v>La Web muestra ofertas reales y su expiresAt. • Permite aceptar/rechazar mediante los endpoints reales. • La aceptación transfiere la cita existente. • El rechazo no crea una cita. • El cliente no recalcula elegibilidad ni ranking.</x:v>
       </x:c>
       <x:c r="L26" t="str">
-        <x:v>feat/web-reassignment-offers · validación técnica y manual PASS</x:v>
+        <x:v>feat/web-reassignment-offers · PR #93 · merge 5701ab7</x:v>
       </x:c>
       <x:c r="M26" t="str">
-        <x:v>HU-022 · Done técnico</x:v>
+        <x:v>HU-022 · Done</x:v>
       </x:c>
       <x:c r="N26" t="str">
-        <x:v>Implementación y validación completas: GET /reassignments/offers/me, ruta /ofertas, expiresAt real, aceptar/rechazar, estados finales y seed:reassignment-demo. Prueba manual: expiración visual PASS, ACCEPT transfiere cita AGENDADA y REJECT no crea cita. Pendiente integración administrativa a main.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="15.75" customHeight="1">
-      <x:c r="A27" s="28" t="str">
-        <x:v>Nota: HU-001 a HU-020 mantienen sus Story Points históricos (105 SP). HU-021 y HU-022 fueron incorporadas posteriormente y quedan Por estimar hasta Refinement/Planning.</x:v>
-      </x:c>
-      <x:c r="B27" s="29"/>
-      <x:c r="C27" s="29"/>
-      <x:c r="D27" s="29"/>
-      <x:c r="E27" s="29"/>
-      <x:c r="F27" s="29"/>
-      <x:c r="G27" s="29"/>
-      <x:c r="H27" s="29"/>
-      <x:c r="I27" s="29"/>
-      <x:c r="J27" s="29"/>
-      <x:c r="K27" s="29"/>
-      <x:c r="L27" s="29"/>
-      <x:c r="M27" s="29"/>
-      <x:c r="N27" s="29"/>
-    </x:row>
-    <x:row r="28" ht="15.75" customHeight="1">
-      <x:c r="A28" s="29"/>
-      <x:c r="B28" s="29"/>
-      <x:c r="C28" s="29"/>
-      <x:c r="D28" s="29"/>
-      <x:c r="E28" s="29"/>
-      <x:c r="F28" s="29"/>
-      <x:c r="G28" s="29"/>
-      <x:c r="H28" s="29"/>
-      <x:c r="I28" s="29"/>
-      <x:c r="J28" s="29"/>
-      <x:c r="K28" s="29"/>
-      <x:c r="L28" s="29"/>
-      <x:c r="M28" s="29"/>
-      <x:c r="N28" s="29"/>
-    </x:row>
-    <x:row r="29" ht="15.75" customHeight="1"/>
+        <x:v>Validación completa Web + API + PostgreSQL: ACCEPT transfirió cita AGENDADA; REJECT no creó cita; oferta vencida deshabilitada sin mutación desde el cliente.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="70" customHeight="1">
+      <x:c r="A27" s="55" t="str">
+        <x:v>HU-023</x:v>
+      </x:c>
+      <x:c r="B27" s="57" t="str">
+        <x:v>Ofertas / Reasignación</x:v>
+      </x:c>
+      <x:c r="C27" s="57" t="str">
+        <x:v>Como sistema CitaJusta, quiero expirar automáticamente las ofertas vencidas y continuar con el siguiente candidato elegible, para recuperar cupos liberados sin depender de intervención manual.</x:v>
+      </x:c>
+      <x:c r="D27" s="57" t="str">
+        <x:v>Automatizar expiración y continuidad de reasignación</x:v>
+      </x:c>
+      <x:c r="E27" s="57" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F27" s="57" t="str">
+        <x:v>Por estimar</x:v>
+      </x:c>
+      <x:c r="G27" s="57" t="str">
+        <x:v>Sprint 6</x:v>
+      </x:c>
+      <x:c r="H27" s="57" t="str">
+        <x:v>Crítica</x:v>
+      </x:c>
+      <x:c r="I27" s="57" t="str">
+        <x:v>RF-029 / RF-030 / RF-036</x:v>
+      </x:c>
+      <x:c r="J27" s="57" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="K27" s="57" t="str">
+        <x:v>Una oferta PENDING vencida pasa de forma persistente a EXPIRED. • La continuidad genera como máximo una siguiente oferta. • Sin candidatos el proceso queda EXHAUSTED. • Cupo/contexto inutilizable cierra CANCELLED. • La operación es idempotente, transaccional y segura ante concurrencia.</x:v>
+      </x:c>
+      <x:c r="L27" s="57" t="str">
+        <x:v>feat/automatic-offer-expiration · PR #96 · merge 109b1c9</x:v>
+      </x:c>
+      <x:c r="M27" s="57" t="str">
+        <x:v>HU-023 · Done</x:v>
+      </x:c>
+      <x:c r="N27" s="57" t="str">
+        <x:v>Runner interno sin dependencias nuevas. Auditoría OFFER_EXPIRED. Validación: API 368/368; E2E expiración 10/10; reasignaciones 20/20; audit 11/11; policy 13/13; reports 15/15; checkpoint 1/1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="70" customHeight="1">
+      <x:c r="A28" s="57" t="str">
+        <x:v>HU-024</x:v>
+      </x:c>
+      <x:c r="B28" s="57" t="str">
+        <x:v>Notificaciones</x:v>
+      </x:c>
+      <x:c r="C28" s="57" t="str">
+        <x:v>Como usuario de CitaJusta, quiero recibir y consultar notificaciones internas sobre eventos importantes de mis citas, lista de espera y ofertas, para mantenerme informado sin depender de servicios externos.</x:v>
+      </x:c>
+      <x:c r="D28" s="57" t="str">
+        <x:v>Implementar notificaciones internas</x:v>
+      </x:c>
+      <x:c r="E28" s="57" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F28" s="57" t="str">
+        <x:v>Por estimar</x:v>
+      </x:c>
+      <x:c r="G28" s="57" t="str">
+        <x:v>Sprint 6</x:v>
+      </x:c>
+      <x:c r="H28" s="57" t="str">
+        <x:v>Alta</x:v>
+      </x:c>
+      <x:c r="I28" s="57" t="str">
+        <x:v>RF-034</x:v>
+      </x:c>
+      <x:c r="J28" s="57" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="K28" s="57" t="str">
+        <x:v>Las notificaciones se persisten dentro de las transacciones reales del dominio. • Sólo el destinatario autenticado puede consultarlas o marcarlas como leídas. • Reintentos idempotentes no generan duplicados. • La Web muestra contador, listado y lectura persistente.</x:v>
+      </x:c>
+      <x:c r="L28" s="57" t="str">
+        <x:v>feat/internal-notifications · PR #99 · merge b1bff30</x:v>
+      </x:c>
+      <x:c r="M28" s="57" t="str">
+        <x:v>HU-024 · Done</x:v>
+      </x:c>
+      <x:c r="N28" s="57" t="str">
+        <x:v>Ocho eventos integrados. API /notifications/me + unread-count + read. Web /notificaciones. Validación: nuevos API 6/6; E2E notifications 8/8; API dirigida 157/157; regresión crítica 87/87; Web 83/83; prueba manual de lectura y logout/login PASS.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
+      <x:c r="A29" t="str">
+        <x:v>Nota: HU-001 a HU-020 mantienen sus Story Points históricos (105 SP). HU-021 a HU-024 quedan Por estimar hasta Refinement/Planning. El estado Done refleja implementación, pruebas y trazabilidad verificable en GitHub.</x:v>
+      </x:c>
+      <x:c r="B29"/>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
+      <x:c r="E29"/>
+      <x:c r="F29"/>
+      <x:c r="G29"/>
+      <x:c r="H29"/>
+      <x:c r="I29"/>
+      <x:c r="J29"/>
+      <x:c r="K29"/>
+      <x:c r="L29"/>
+      <x:c r="M29"/>
+      <x:c r="N29"/>
+    </x:row>
     <x:row r="30" ht="15.75" customHeight="1"/>
     <x:row r="31" ht="15.75" customHeight="1"/>
     <x:row r="32" ht="15.75" customHeight="1"/>
@@ -3363,7 +3500,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
     <x:mergeCell ref="A2:N2"/>
-    <x:mergeCell ref="A27:N28"/>
+    <x:mergeCell ref="A29:N29"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="E5:E24">
     <x:cfRule type="expression" dxfId="4" priority="1">
@@ -3395,7 +3532,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a21b0c75bf9454d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf053b8e3fbc0407a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3411,7 +3548,7 @@
   <x:sheetData>
     <x:row r="1" ht="27.75" customHeight="1">
       <x:c r="A1" s="8" t="str">
-        <x:v>CITAJUSTA — RESUMEN DEL PRODUCT BACKLOG (ACTUALIZADO 20-09-2026)</x:v>
+        <x:v>CITAJUSTA — RESUMEN DEL PRODUCT BACKLOG (ACTUALIZADO 21-09-2026)</x:v>
       </x:c>
       <x:c r="B1" s="9"/>
       <x:c r="C1" s="9"/>
@@ -3440,7 +3577,7 @@
         <x:v>Historias totales</x:v>
       </x:c>
       <x:c r="B4" s="1" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C4" s="3"/>
       <x:c r="D4" s="5" t="str">
@@ -3448,7 +3585,7 @@
       </x:c>
       <x:c r="E4" s="5" t="n">
         <x:f t="shared" ref="E4:E6" si="0">B6</x:f>
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F4" s="3"/>
     </x:row>
@@ -3474,7 +3611,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B6" s="1" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C6" s="3"/>
       <x:c r="D6" s="5" t="str">
@@ -3551,7 +3688,7 @@
         <x:v>Historias MVP</x:v>
       </x:c>
       <x:c r="B11" s="5" t="n">
-        <x:v>18</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C11" s="3"/>
       <x:c r="D11" s="5" t="str">
@@ -3574,7 +3711,7 @@
         <x:v>Sprint 6</x:v>
       </x:c>
       <x:c r="E12" s="5" t="n">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F12" s="5"/>
     </x:row>
@@ -3598,7 +3735,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="E14" s="5" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F14" s="5"/>
     </x:row>
@@ -3619,11 +3756,11 @@
     <x:row r="16">
       <x:c r="A16" s="14" t="str">
         <x:v>• Backend HU-001 a HU-020 completado.
-• HU-021 Web de lista de espera/preferencias completada y mergeada mediante PR #89.
-• HU-022 Web de ofertas/reasignación completada técnicamente en feat/web-reassignment-offers.
-• Validación HU-022: Web 71/71, pruebas enfocadas 10/10 y E2E reales de reasignación 20/20; build API/Web, Prisma validate y check:dev PASS.
-• Prueba manual: oferta vencida sin mutación, ACCEPT con cita AGENDADA transferida y REJECT sin cita para el destinatario.
-• Story Points de HU-021/HU-022 quedan Por estimar; el 100% de los 105 SP históricos HU-001–HU-020 está completado.</x:v>
+• HU-021 Web waitlist/preferencias Done (PR #89, merge c291d17).
+• HU-022 Web ofertas Done (PR #93, merge 5701ab7).
+• HU-023 expiración automática/continuidad Done (PR #96, merge 109b1c9).
+• HU-024 notificaciones internas Done (PR #99, merge b1bff30).
+• RF-029/RF-030/RF-034 cubiertos. HU-021 a HU-024 mantienen Story Points Por estimar.</x:v>
       </x:c>
       <x:c r="B16" s="15"/>
       <x:c r="C16" s="7"/>
@@ -3680,7 +3817,7 @@
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>HU-022 quedó funcionalmente terminada y validada de punta a punta en Web + API + PostgreSQL. La rama feat/web-reassignment-offers queda lista para commit, PR y merge; después corresponde actualizar el estado visual del Kanban.</x:v>
+        <x:v>HU-024 quedó completada y validada con notificaciones persistentes, deduplicación transaccional, API autenticada y centro Web /notificaciones. El núcleo de reasignación ya incluye expiración automática y continuidad segura mediante HU-023.</x:v>
       </x:c>
       <x:c r="B24" s="22"/>
       <x:c r="C24" s="22"/>
@@ -4694,6 +4831,6 @@
     <x:mergeCell ref="A24:F27"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e9bd541bc094adb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38509467ac3443b6"/>
 </x:worksheet>
 </file>
</xml_diff>